<commit_message>
FIX on user import
</commit_message>
<xml_diff>
--- a/test/fixtures/business sites 1.xlsx
+++ b/test/fixtures/business sites 1.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26605"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1da6715471b04c19/Energiepad/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B547E9F5-21B0-4CB4-BD49-6188F152F873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{59ECF548-5CAE-412A-B12F-03F73E5801D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main Contact" sheetId="1" r:id="rId1"/>
     <sheet name="Sites" sheetId="2" r:id="rId2"/>
-    <sheet name="O &amp; S" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
   <si>
     <t>businessName</t>
   </si>
@@ -173,39 +172,6 @@
   </si>
   <si>
     <t>Newcastle</t>
-  </si>
-  <si>
-    <t>Operation and Setpoints</t>
-  </si>
-  <si>
-    <t>Energy  Demand</t>
-  </si>
-  <si>
-    <t>Start Date</t>
-  </si>
-  <si>
-    <t>End Date</t>
-  </si>
-  <si>
-    <t>Temperature set point</t>
-  </si>
-  <si>
-    <t>Days in the year</t>
-  </si>
-  <si>
-    <t>Heating</t>
-  </si>
-  <si>
-    <t>Cooling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lighting </t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Powering</t>
   </si>
 </sst>
 </file>
@@ -215,18 +181,11 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -247,27 +206,6 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -297,30 +235,20 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -630,7 +558,7 @@
       <c r="G2" s="5">
         <v>447866666</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="7" t="s">
         <v>22</v>
       </c>
       <c r="I2" s="4" t="s">
@@ -2740,251 +2668,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F800EC39-B777-41D4-B1AD-85C9BFA0246E}">
-  <dimension ref="A1:K16"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="13.28515625" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11">
-      <c r="C1" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" s="3">
-        <v>45047</v>
-      </c>
-      <c r="D3" s="3">
-        <v>45199</v>
-      </c>
-      <c r="E3" s="11">
-        <v>18</v>
-      </c>
-      <c r="F3" s="11">
-        <f>D3-C3</f>
-        <v>152</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="A4" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C4" s="3">
-        <v>45200</v>
-      </c>
-      <c r="D4" s="3">
-        <v>45412</v>
-      </c>
-      <c r="E4" s="11">
-        <v>16</v>
-      </c>
-      <c r="F4" s="11">
-        <f>D4-C4</f>
-        <v>212</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" t="s">
-        <v>53</v>
-      </c>
-      <c r="C5" s="7">
-        <v>44927</v>
-      </c>
-      <c r="D5" s="7">
-        <v>45291</v>
-      </c>
-      <c r="E5" t="s">
-        <v>54</v>
-      </c>
-      <c r="F5" s="11">
-        <f>D5-C5</f>
-        <v>364</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" s="7">
-        <v>44927</v>
-      </c>
-      <c r="D6" s="7">
-        <v>45291</v>
-      </c>
-      <c r="E6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="11">
-        <f>D6-C6</f>
-        <v>364</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
-      <c r="A7" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="3">
-        <v>45047</v>
-      </c>
-      <c r="D7" s="3">
-        <v>45199</v>
-      </c>
-      <c r="E7" s="11">
-        <v>18</v>
-      </c>
-      <c r="F7" s="11">
-        <f>D7-C7</f>
-        <v>152</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
-      <c r="A8" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="3">
-        <v>45200</v>
-      </c>
-      <c r="D8" s="3">
-        <v>45412</v>
-      </c>
-      <c r="E8" s="11">
-        <v>16</v>
-      </c>
-      <c r="F8" s="11">
-        <f>D8-C8</f>
-        <v>212</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
-      <c r="A9" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" t="s">
-        <v>53</v>
-      </c>
-      <c r="C9" s="7">
-        <v>44927</v>
-      </c>
-      <c r="D9" s="7">
-        <v>45291</v>
-      </c>
-      <c r="E9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F9" s="11">
-        <f>D9-C9</f>
-        <v>364</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
-      <c r="A10" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="B10" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" s="7">
-        <v>44927</v>
-      </c>
-      <c r="D10" s="7">
-        <v>45291</v>
-      </c>
-      <c r="E10" t="s">
-        <v>54</v>
-      </c>
-      <c r="F10" s="11">
-        <f>D10-C10</f>
-        <v>364</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
-      <c r="A11" s="11"/>
-    </row>
-    <row r="13" spans="1:11">
-      <c r="K13" s="11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11">
-      <c r="K14" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11">
-      <c r="K15" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11">
-      <c r="K16" s="11" t="s">
-        <v>55</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="C1:F1"/>
-  </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B10" xr:uid="{EAAD6D50-D0F2-4660-BD5E-90AC4BDBA33F}">
-      <formula1>$K$13:$K$16</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
FIX on sites import
</commit_message>
<xml_diff>
--- a/test/fixtures/business sites 1.xlsx
+++ b/test/fixtures/business sites 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91983\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D492D1C8-5044-45AD-8027-F2856BBE1F35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{034ECB9C-4319-4D6B-AF7D-D181A441CB60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Business" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="409">
   <si>
     <t>Business Name</t>
   </si>
@@ -126,9 +126,6 @@
     <t>EUR</t>
   </si>
   <si>
-    <t>Site Code</t>
-  </si>
-  <si>
     <t>Site Name</t>
   </si>
   <si>
@@ -147,9 +144,6 @@
     <t>FTE Working Hours/Day</t>
   </si>
   <si>
-    <t>Site 001</t>
-  </si>
-  <si>
     <t>Corporate</t>
   </si>
   <si>
@@ -159,7 +153,7 @@
     <t xml:space="preserve">London </t>
   </si>
   <si>
-    <t>Site 002</t>
+    <t>Kazakhstan</t>
   </si>
   <si>
     <t>Regional Office</t>
@@ -168,12 +162,12 @@
     <t>2 Leyton Street</t>
   </si>
   <si>
+    <t>Newcastle</t>
+  </si>
+  <si>
     <t>NE12 7BH</t>
   </si>
   <si>
-    <t>Newcastle</t>
-  </si>
-  <si>
     <t>Administraive and Support Service Activities</t>
   </si>
   <si>
@@ -688,9 +682,6 @@
   </si>
   <si>
     <t>GYD</t>
-  </si>
-  <si>
-    <t>Kazakhstan</t>
   </si>
   <si>
     <t>HTG</t>
@@ -2672,38 +2663,40 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J1000"/>
+  <dimension ref="A1:I1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" customWidth="1"/>
-    <col min="5" max="8" width="8.7109375" customWidth="1"/>
-    <col min="9" max="9" width="23" customWidth="1"/>
-    <col min="10" max="28" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="19.28515625" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" customWidth="1"/>
+    <col min="3" max="4" width="13.42578125" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" customWidth="1"/>
+    <col min="6" max="7" width="8.7109375" customWidth="1"/>
+    <col min="8" max="8" width="23" customWidth="1"/>
+    <col min="9" max="9" width="21.140625" customWidth="1"/>
+    <col min="10" max="27" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="14.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>31</v>
@@ -2711,72 +2704,63 @@
       <c r="I1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="J1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="14.25">
-      <c r="A2" t="s">
+      <c r="C2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>24</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" s="1">
+        <v>500</v>
+      </c>
+      <c r="H2" s="1">
+        <v>8</v>
+      </c>
+      <c r="I2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="15" customHeight="1">
+      <c r="A3" t="s">
         <v>37</v>
       </c>
-      <c r="G2" s="1">
-        <v>300</v>
-      </c>
-      <c r="H2" s="1">
-        <v>500</v>
-      </c>
-      <c r="I2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="1">
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3">
+        <v>400</v>
+      </c>
+      <c r="H3">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" ht="15" customHeight="1">
-      <c r="A3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G3">
-        <v>200</v>
-      </c>
-      <c r="H3">
-        <v>400</v>
-      </c>
-      <c r="I3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3">
-        <v>8</v>
+      <c r="I3">
+        <v>4</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -3760,6 +3744,11 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F3" xr:uid="{120F0D9E-7EBE-44B6-BA50-B43A37C1AB02}">
+      <formula1>countries</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
@@ -3776,35 +3765,35 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" t="s">
         <v>43</v>
-      </c>
-      <c r="C1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F2" t="s">
         <v>46</v>
-      </c>
-      <c r="C2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s">
         <v>25</v>
       </c>
       <c r="F3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -3812,18 +3801,18 @@
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F5" t="s">
         <v>26</v>
@@ -3831,98 +3820,98 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" t="s">
         <v>57</v>
-      </c>
-      <c r="C7" t="s">
-        <v>58</v>
-      </c>
-      <c r="F7" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F10" t="s">
         <v>64</v>
-      </c>
-      <c r="C10" t="s">
-        <v>65</v>
-      </c>
-      <c r="F10" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F11" t="s">
         <v>67</v>
-      </c>
-      <c r="C11" t="s">
-        <v>68</v>
-      </c>
-      <c r="F11" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" t="s">
         <v>70</v>
-      </c>
-      <c r="C12" t="s">
-        <v>71</v>
-      </c>
-      <c r="F12" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" t="s">
         <v>73</v>
-      </c>
-      <c r="C13" t="s">
-        <v>74</v>
-      </c>
-      <c r="F13" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F14" t="s">
         <v>26</v>
@@ -3930,13 +3919,13 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" t="s">
         <v>78</v>
-      </c>
-      <c r="C15" t="s">
-        <v>79</v>
-      </c>
-      <c r="F15" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -3944,62 +3933,62 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F16" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
+        <v>81</v>
+      </c>
+      <c r="C17" t="s">
+        <v>82</v>
+      </c>
+      <c r="F17" t="s">
         <v>83</v>
-      </c>
-      <c r="C17" t="s">
-        <v>84</v>
-      </c>
-      <c r="F17" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" t="s">
+        <v>85</v>
+      </c>
+      <c r="F18" t="s">
         <v>86</v>
-      </c>
-      <c r="C18" t="s">
-        <v>87</v>
-      </c>
-      <c r="F18" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" t="s">
+        <v>88</v>
+      </c>
+      <c r="F19" t="s">
         <v>89</v>
-      </c>
-      <c r="C19" t="s">
-        <v>90</v>
-      </c>
-      <c r="F19" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" t="s">
+        <v>91</v>
+      </c>
+      <c r="F20" t="s">
         <v>92</v>
-      </c>
-      <c r="C20" t="s">
-        <v>93</v>
-      </c>
-      <c r="F20" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C21" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F21" t="s">
         <v>26</v>
@@ -4007,269 +3996,269 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" t="s">
+        <v>96</v>
+      </c>
+      <c r="F22" t="s">
         <v>97</v>
-      </c>
-      <c r="C22" t="s">
-        <v>98</v>
-      </c>
-      <c r="F22" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
+        <v>98</v>
+      </c>
+      <c r="C23" t="s">
+        <v>99</v>
+      </c>
+      <c r="F23" t="s">
         <v>100</v>
-      </c>
-      <c r="C23" t="s">
-        <v>101</v>
-      </c>
-      <c r="F23" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="C24" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="C25" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F25" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="C26" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F26" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="C27" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F27" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="C28" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F28" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="C29" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F29" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="C30" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F30" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="C31" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F31" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="C32" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F32" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="33" spans="3:6">
       <c r="C33" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F33" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="34" spans="3:6">
       <c r="C34" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F34" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="3:6">
       <c r="C35" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F35" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="36" spans="3:6">
       <c r="C36" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F36" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="37" spans="3:6">
       <c r="C37" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F37" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="38" spans="3:6">
       <c r="C38" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F38" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="39" spans="3:6">
       <c r="C39" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F39" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="40" spans="3:6">
       <c r="C40" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F40" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="41" spans="3:6">
       <c r="C41" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="42" spans="3:6">
       <c r="C42" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F42" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="43" spans="3:6">
       <c r="C43" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F43" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="44" spans="3:6">
       <c r="C44" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F44" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="45" spans="3:6">
       <c r="C45" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F45" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="46" spans="3:6">
       <c r="C46" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F46" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="47" spans="3:6">
       <c r="C47" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F47" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="48" spans="3:6">
       <c r="C48" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F48" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="49" spans="3:6">
       <c r="C49" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F49" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="50" spans="3:6">
       <c r="C50" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F50" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="51" spans="3:6">
       <c r="C51" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F51" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="52" spans="3:6">
       <c r="C52" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F52" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="53" spans="3:6">
       <c r="C53" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F53" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="54" spans="3:6">
       <c r="C54" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="F54" t="s">
         <v>26</v>
@@ -4277,103 +4266,103 @@
     </row>
     <row r="55" spans="3:6">
       <c r="C55" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F55" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="56" spans="3:6">
       <c r="C56" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F56" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="57" spans="3:6">
       <c r="C57" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F57" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="58" spans="3:6">
       <c r="C58" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F58" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="59" spans="3:6">
       <c r="C59" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F59" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="60" spans="3:6">
       <c r="C60" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F60" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="61" spans="3:6">
       <c r="C61" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F61" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="62" spans="3:6">
       <c r="C62" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F62" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="63" spans="3:6">
       <c r="C63" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F63" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="64" spans="3:6">
       <c r="C64" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F64" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="65" spans="3:6">
       <c r="C65" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F65" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="66" spans="3:6">
       <c r="C66" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F66" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="67" spans="3:6">
       <c r="C67" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F67" t="s">
         <v>26</v>
@@ -4381,39 +4370,39 @@
     </row>
     <row r="68" spans="3:6">
       <c r="C68" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F68" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="69" spans="3:6">
       <c r="C69" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="F69" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="70" spans="3:6">
       <c r="C70" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F70" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="71" spans="3:6">
       <c r="C71" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F71" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="72" spans="3:6">
       <c r="C72" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="F72" t="s">
         <v>26</v>
@@ -4421,7 +4410,7 @@
     </row>
     <row r="73" spans="3:6">
       <c r="C73" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F73" t="s">
         <v>26</v>
@@ -4429,7 +4418,7 @@
     </row>
     <row r="74" spans="3:6">
       <c r="C74" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F74" t="s">
         <v>26</v>
@@ -4437,15 +4426,15 @@
     </row>
     <row r="75" spans="3:6">
       <c r="C75" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F75" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="76" spans="3:6">
       <c r="C76" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F76" t="s">
         <v>26</v>
@@ -4453,31 +4442,31 @@
     </row>
     <row r="77" spans="3:6">
       <c r="C77" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F77" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="78" spans="3:6">
       <c r="C78" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F78" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="79" spans="3:6">
       <c r="C79" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F79" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="80" spans="3:6">
       <c r="C80" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F80" t="s">
         <v>26</v>
@@ -4485,23 +4474,23 @@
     </row>
     <row r="81" spans="3:6">
       <c r="C81" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F81" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="82" spans="3:6">
       <c r="C82" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F82" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="83" spans="3:6">
       <c r="C83" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F83" t="s">
         <v>26</v>
@@ -4509,23 +4498,23 @@
     </row>
     <row r="84" spans="3:6">
       <c r="C84" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F84" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="85" spans="3:6">
       <c r="C85" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F85" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="86" spans="3:6">
       <c r="C86" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F86" t="s">
         <v>26</v>
@@ -4533,63 +4522,63 @@
     </row>
     <row r="87" spans="3:6">
       <c r="C87" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F87" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="88" spans="3:6">
       <c r="C88" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F88" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="89" spans="3:6">
       <c r="C89" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F89" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="90" spans="3:6">
       <c r="C90" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F90" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="91" spans="3:6">
       <c r="C91" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F91" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="92" spans="3:6">
       <c r="C92" t="s">
-        <v>215</v>
+        <v>36</v>
       </c>
       <c r="F92" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="93" spans="3:6">
       <c r="C93" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="F93" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="94" spans="3:6">
       <c r="C94" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="F94" t="s">
         <v>26</v>
@@ -4597,71 +4586,71 @@
     </row>
     <row r="95" spans="3:6">
       <c r="C95" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="F95" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
     </row>
     <row r="96" spans="3:6">
       <c r="C96" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="F96" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="97" spans="3:6">
       <c r="C97" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="F97" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
     <row r="98" spans="3:6">
       <c r="C98" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="F98" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="99" spans="3:6">
       <c r="C99" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="F99" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="100" spans="3:6">
       <c r="C100" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="F100" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
     </row>
     <row r="101" spans="3:6">
       <c r="C101" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="F101" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="102" spans="3:6">
       <c r="C102" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="F102" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="103" spans="3:6">
       <c r="C103" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="F103" t="s">
         <v>26</v>
@@ -4669,15 +4658,15 @@
     </row>
     <row r="104" spans="3:6">
       <c r="C104" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="F104" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="105" spans="3:6">
       <c r="C105" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="F105" t="s">
         <v>26</v>
@@ -4685,143 +4674,143 @@
     </row>
     <row r="106" spans="3:6">
       <c r="C106" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="F106" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="107" spans="3:6">
       <c r="C107" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="F107" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="108" spans="3:6">
       <c r="C108" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="F108" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="109" spans="3:6">
       <c r="C109" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="F109" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="110" spans="3:6">
       <c r="C110" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="F110" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
     <row r="111" spans="3:6">
       <c r="C111" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="F111" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="112" spans="3:6">
       <c r="C112" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="F112" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="113" spans="3:6">
       <c r="C113" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="F113" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="114" spans="3:6">
       <c r="C114" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="F114" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="115" spans="3:6">
       <c r="C115" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="F115" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="116" spans="3:6">
       <c r="C116" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="F116" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="117" spans="3:6">
       <c r="C117" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="F117" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
     <row r="118" spans="3:6">
       <c r="C118" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F118" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="119" spans="3:6">
       <c r="C119" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="F119" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="120" spans="3:6">
       <c r="C120" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="F120" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="121" spans="3:6">
       <c r="C121" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="F121" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="122" spans="3:6">
       <c r="C122" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="F122" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
     </row>
     <row r="123" spans="3:6">
       <c r="C123" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="F123" t="s">
         <v>26</v>
@@ -4829,63 +4818,63 @@
     </row>
     <row r="124" spans="3:6">
       <c r="C124" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="F124" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
     </row>
     <row r="125" spans="3:6">
       <c r="C125" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="F125" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
     </row>
     <row r="126" spans="3:6">
       <c r="C126" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="F126" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="127" spans="3:6">
       <c r="C127" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="F127" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="128" spans="3:6">
       <c r="C128" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="F128" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="129" spans="3:6">
       <c r="C129" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="F129" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="130" spans="3:6">
       <c r="C130" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="F130" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="131" spans="3:6">
       <c r="C131" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="F131" t="s">
         <v>26</v>
@@ -4893,15 +4882,15 @@
     </row>
     <row r="132" spans="3:6">
       <c r="C132" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="F132" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="133" spans="3:6">
       <c r="C133" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="F133" t="s">
         <v>26</v>
@@ -4909,23 +4898,23 @@
     </row>
     <row r="134" spans="3:6">
       <c r="C134" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="F134" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="135" spans="3:6">
       <c r="C135" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="F135" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="136" spans="3:6">
       <c r="C136" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F136" t="s">
         <v>26</v>
@@ -4933,31 +4922,31 @@
     </row>
     <row r="137" spans="3:6">
       <c r="C137" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="F137" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
     </row>
     <row r="138" spans="3:6">
       <c r="C138" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F138" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="139" spans="3:6">
       <c r="C139" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="F139" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
     </row>
     <row r="140" spans="3:6">
       <c r="C140" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F140" t="s">
         <v>26</v>
@@ -4965,71 +4954,71 @@
     </row>
     <row r="141" spans="3:6">
       <c r="C141" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="F141" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
     </row>
     <row r="142" spans="3:6">
       <c r="C142" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="F142" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="143" spans="3:6">
       <c r="C143" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="F143" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="144" spans="3:6">
       <c r="C144" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="F144" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
     </row>
     <row r="145" spans="3:6">
       <c r="C145" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="F145" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="146" spans="3:6">
       <c r="C146" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F146" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
     </row>
     <row r="147" spans="3:6">
       <c r="C147" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="F147" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="148" spans="3:6">
       <c r="C148" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="F148" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="149" spans="3:6">
       <c r="C149" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="F149" t="s">
         <v>26</v>
@@ -5037,191 +5026,191 @@
     </row>
     <row r="150" spans="3:6">
       <c r="C150" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="F150" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
     </row>
     <row r="151" spans="3:6">
       <c r="C151" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="F151" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="152" spans="3:6">
       <c r="C152" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="F152" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="153" spans="3:6">
       <c r="C153" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="F153" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
     </row>
     <row r="154" spans="3:6">
       <c r="C154" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="F154" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="155" spans="3:6">
       <c r="C155" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="F155" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
     </row>
     <row r="156" spans="3:6">
       <c r="C156" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="F156" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="157" spans="3:6">
       <c r="C157" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="F157" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="158" spans="3:6">
       <c r="C158" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="F158" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="159" spans="3:6">
       <c r="C159" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="F159" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="160" spans="3:6">
       <c r="C160" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="F160" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="161" spans="3:6">
       <c r="C161" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="F161" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="162" spans="3:6">
       <c r="C162" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="F162" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="163" spans="3:6">
       <c r="C163" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="F163" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="164" spans="3:6">
       <c r="C164" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="F164" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="165" spans="3:6">
       <c r="C165" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="F165" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
     </row>
     <row r="166" spans="3:6">
       <c r="C166" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="F166" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
     </row>
     <row r="167" spans="3:6">
       <c r="C167" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="F167" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
     </row>
     <row r="168" spans="3:6">
       <c r="C168" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="F168" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
     </row>
     <row r="169" spans="3:6">
       <c r="C169" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="F169" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
     </row>
     <row r="170" spans="3:6">
       <c r="C170" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="F170" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
     </row>
     <row r="171" spans="3:6">
       <c r="C171" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="F171" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="172" spans="3:6">
       <c r="C172" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F172" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
     </row>
     <row r="173" spans="3:6">
       <c r="C173" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="F173" t="s">
         <v>26</v>
@@ -5229,23 +5218,23 @@
     </row>
     <row r="174" spans="3:6">
       <c r="C174" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F174" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="175" spans="3:6">
       <c r="C175" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="F175" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
     </row>
     <row r="176" spans="3:6">
       <c r="C176" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="F176" t="s">
         <v>26</v>
@@ -5253,55 +5242,55 @@
     </row>
     <row r="177" spans="3:6">
       <c r="C177" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="F177" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
     </row>
     <row r="178" spans="3:6">
       <c r="C178" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="F178" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
     </row>
     <row r="179" spans="3:6">
       <c r="C179" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="F179" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="180" spans="3:6">
       <c r="C180" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="F180" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
     </row>
     <row r="181" spans="3:6">
       <c r="C181" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="F181" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="182" spans="3:6">
       <c r="C182" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="F182" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="183" spans="3:6">
       <c r="C183" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="F183" t="s">
         <v>26</v>
@@ -5309,23 +5298,23 @@
     </row>
     <row r="184" spans="3:6">
       <c r="C184" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="F184" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="185" spans="3:6">
       <c r="C185" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="F185" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
     </row>
     <row r="186" spans="3:6">
       <c r="C186" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="F186" t="s">
         <v>26</v>
@@ -5333,57 +5322,57 @@
     </row>
     <row r="187" spans="3:6">
       <c r="C187" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="F187" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
     </row>
     <row r="188" spans="3:6">
       <c r="C188" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="F188" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
     </row>
     <row r="189" spans="3:6">
       <c r="C189" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="F189" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="190" spans="3:6">
       <c r="C190" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="F190" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="191" spans="3:6">
       <c r="C191" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="F191" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="192" spans="3:6">
       <c r="F192" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="193" spans="6:6">
       <c r="F193" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
     </row>
     <row r="194" spans="6:6">
       <c r="F194" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
     </row>
     <row r="195" spans="6:6">
@@ -5398,32 +5387,32 @@
     </row>
     <row r="197" spans="6:6">
       <c r="F197" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
     <row r="198" spans="6:6">
       <c r="F198" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
     </row>
     <row r="199" spans="6:6">
       <c r="F199" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="200" spans="6:6">
       <c r="F200" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="201" spans="6:6">
       <c r="F201" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
     <row r="202" spans="6:6">
       <c r="F202" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="203" spans="6:6">
@@ -5433,202 +5422,202 @@
     </row>
     <row r="204" spans="6:6">
       <c r="F204" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
     <row r="205" spans="6:6">
       <c r="F205" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="206" spans="6:6">
       <c r="F206" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
     </row>
     <row r="207" spans="6:6">
       <c r="F207" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="208" spans="6:6">
       <c r="F208" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="209" spans="6:6">
       <c r="F209" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
     </row>
     <row r="210" spans="6:6">
       <c r="F210" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="211" spans="6:6">
       <c r="F211" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="212" spans="6:6">
       <c r="F212" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="213" spans="6:6">
       <c r="F213" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="214" spans="6:6">
       <c r="F214" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
     <row r="215" spans="6:6">
       <c r="F215" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
     <row r="216" spans="6:6">
       <c r="F216" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="217" spans="6:6">
       <c r="F217" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="218" spans="6:6">
       <c r="F218" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="219" spans="6:6">
       <c r="F219" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="220" spans="6:6">
       <c r="F220" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="221" spans="6:6">
       <c r="F221" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="222" spans="6:6">
       <c r="F222" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
     <row r="223" spans="6:6">
       <c r="F223" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="224" spans="6:6">
       <c r="F224" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="225" spans="6:6">
       <c r="F225" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
     </row>
     <row r="226" spans="6:6">
       <c r="F226" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="227" spans="6:6">
       <c r="F227" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
     </row>
     <row r="228" spans="6:6">
       <c r="F228" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="229" spans="6:6">
       <c r="F229" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="230" spans="6:6">
       <c r="F230" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="231" spans="6:6">
       <c r="F231" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
     <row r="232" spans="6:6">
       <c r="F232" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="233" spans="6:6">
       <c r="F233" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="234" spans="6:6">
       <c r="F234" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="235" spans="6:6">
       <c r="F235" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="236" spans="6:6">
       <c r="F236" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="237" spans="6:6">
       <c r="F237" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="238" spans="6:6">
       <c r="F238" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="239" spans="6:6">
       <c r="F239" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="240" spans="6:6">
       <c r="F240" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="241" spans="6:6">
       <c r="F241" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="242" spans="6:6">
       <c r="F242" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
     </row>
     <row r="243" spans="6:6">
       <c r="F243" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
REFACTOR on business,sites import
</commit_message>
<xml_diff>
--- a/test/fixtures/business sites 1.xlsx
+++ b/test/fixtures/business sites 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26616"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91983\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{034ECB9C-4319-4D6B-AF7D-D181A441CB60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7FDDD39-7C2E-4FC1-9F45-8EC05F95757B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Business" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="412">
   <si>
     <t>Business Name</t>
   </si>
@@ -126,6 +126,9 @@
     <t>EUR</t>
   </si>
   <si>
+    <t>Site Code</t>
+  </si>
+  <si>
     <t>Site Name</t>
   </si>
   <si>
@@ -144,6 +147,9 @@
     <t>FTE Working Hours/Day</t>
   </si>
   <si>
+    <t>head_office</t>
+  </si>
+  <si>
     <t>Corporate</t>
   </si>
   <si>
@@ -154,6 +160,9 @@
   </si>
   <si>
     <t>Kazakhstan</t>
+  </si>
+  <si>
+    <t>regional_office</t>
   </si>
   <si>
     <t>Regional Office</t>
@@ -2663,40 +2672,41 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I1000"/>
+  <dimension ref="A1:J1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" customWidth="1"/>
-    <col min="3" max="4" width="13.42578125" customWidth="1"/>
-    <col min="5" max="5" width="15.140625" customWidth="1"/>
-    <col min="6" max="7" width="8.7109375" customWidth="1"/>
-    <col min="8" max="8" width="23" customWidth="1"/>
-    <col min="9" max="9" width="21.140625" customWidth="1"/>
-    <col min="10" max="27" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="5" width="13.42578125" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" customWidth="1"/>
+    <col min="9" max="9" width="23" customWidth="1"/>
+    <col min="10" max="10" width="21.140625" customWidth="1"/>
+    <col min="11" max="28" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
         <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="F1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>31</v>
@@ -2704,62 +2714,71 @@
       <c r="I1" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="1" t="s">
+      <c r="J1" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="C2" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" s="1">
+        <v>500</v>
+      </c>
+      <c r="I2" s="1">
+        <v>8</v>
+      </c>
+      <c r="J2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15" customHeight="1">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G2" s="1">
-        <v>500</v>
-      </c>
-      <c r="H2" s="1">
+      <c r="D3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3">
+        <v>400</v>
+      </c>
+      <c r="I3">
         <v>8</v>
       </c>
-      <c r="I2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="15" customHeight="1">
-      <c r="A3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3">
-        <v>400</v>
-      </c>
-      <c r="H3">
-        <v>8</v>
-      </c>
-      <c r="I3">
+      <c r="J3">
         <v>4</v>
       </c>
     </row>
@@ -3745,7 +3764,7 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F3" xr:uid="{120F0D9E-7EBE-44B6-BA50-B43A37C1AB02}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G3" xr:uid="{120F0D9E-7EBE-44B6-BA50-B43A37C1AB02}">
       <formula1>countries</formula1>
     </dataValidation>
   </dataValidations>
@@ -3765,35 +3784,35 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C3" t="s">
         <v>25</v>
       </c>
       <c r="F3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -3801,18 +3820,18 @@
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F5" t="s">
         <v>26</v>
@@ -3820,98 +3839,98 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" t="s">
         <v>60</v>
-      </c>
-      <c r="C9" t="s">
-        <v>61</v>
-      </c>
-      <c r="F9" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C10" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C11" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C12" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F12" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C13" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F14" t="s">
         <v>26</v>
@@ -3919,13 +3938,13 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C15" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F15" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -3933,62 +3952,62 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F16" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C17" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F17" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C18" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F18" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C19" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F19" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C20" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F20" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C21" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F21" t="s">
         <v>26</v>
@@ -3996,269 +4015,269 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C22" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F22" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C23" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F23" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="C24" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F24" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="C25" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F25" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="C26" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="F26" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="C27" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="F27" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="C28" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F28" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="C29" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="F29" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="C30" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F30" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="C31" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F31" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="C32" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F32" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="33" spans="3:6">
       <c r="C33" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="F33" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="34" spans="3:6">
       <c r="C34" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F34" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="35" spans="3:6">
       <c r="C35" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F35" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="36" spans="3:6">
       <c r="C36" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F36" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="37" spans="3:6">
       <c r="C37" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F37" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="38" spans="3:6">
       <c r="C38" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="F38" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="39" spans="3:6">
       <c r="C39" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="F39" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="40" spans="3:6">
       <c r="C40" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F40" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="41" spans="3:6">
       <c r="C41" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F41" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="42" spans="3:6">
       <c r="C42" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F42" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="43" spans="3:6">
       <c r="C43" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F43" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="44" spans="3:6">
       <c r="C44" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="F44" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="45" spans="3:6">
       <c r="C45" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F45" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="46" spans="3:6">
       <c r="C46" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="F46" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="47" spans="3:6">
       <c r="C47" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F47" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="48" spans="3:6">
       <c r="C48" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F48" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="49" spans="3:6">
       <c r="C49" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="F49" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="50" spans="3:6">
       <c r="C50" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="F50" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="51" spans="3:6">
       <c r="C51" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F51" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="52" spans="3:6">
       <c r="C52" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F52" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="53" spans="3:6">
       <c r="C53" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F53" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="54" spans="3:6">
       <c r="C54" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="F54" t="s">
         <v>26</v>
@@ -4266,103 +4285,103 @@
     </row>
     <row r="55" spans="3:6">
       <c r="C55" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F55" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="56" spans="3:6">
       <c r="C56" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F56" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="57" spans="3:6">
       <c r="C57" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F57" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="58" spans="3:6">
       <c r="C58" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="F58" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="59" spans="3:6">
       <c r="C59" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="F59" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="60" spans="3:6">
       <c r="C60" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F60" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="61" spans="3:6">
       <c r="C61" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="F61" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="62" spans="3:6">
       <c r="C62" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="F62" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="63" spans="3:6">
       <c r="C63" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F63" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="64" spans="3:6">
       <c r="C64" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="F64" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="65" spans="3:6">
       <c r="C65" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F65" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="66" spans="3:6">
       <c r="C66" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="F66" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="67" spans="3:6">
       <c r="C67" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F67" t="s">
         <v>26</v>
@@ -4370,39 +4389,39 @@
     </row>
     <row r="68" spans="3:6">
       <c r="C68" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="F68" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="69" spans="3:6">
       <c r="C69" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F69" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="70" spans="3:6">
       <c r="C70" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="F70" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="71" spans="3:6">
       <c r="C71" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F71" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="72" spans="3:6">
       <c r="C72" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="F72" t="s">
         <v>26</v>
@@ -4410,7 +4429,7 @@
     </row>
     <row r="73" spans="3:6">
       <c r="C73" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="F73" t="s">
         <v>26</v>
@@ -4418,7 +4437,7 @@
     </row>
     <row r="74" spans="3:6">
       <c r="C74" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F74" t="s">
         <v>26</v>
@@ -4426,15 +4445,15 @@
     </row>
     <row r="75" spans="3:6">
       <c r="C75" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="F75" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="76" spans="3:6">
       <c r="C76" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="F76" t="s">
         <v>26</v>
@@ -4442,31 +4461,31 @@
     </row>
     <row r="77" spans="3:6">
       <c r="C77" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F77" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="78" spans="3:6">
       <c r="C78" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="F78" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="79" spans="3:6">
       <c r="C79" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F79" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="80" spans="3:6">
       <c r="C80" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="F80" t="s">
         <v>26</v>
@@ -4474,23 +4493,23 @@
     </row>
     <row r="81" spans="3:6">
       <c r="C81" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F81" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="82" spans="3:6">
       <c r="C82" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F82" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="83" spans="3:6">
       <c r="C83" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F83" t="s">
         <v>26</v>
@@ -4498,23 +4517,23 @@
     </row>
     <row r="84" spans="3:6">
       <c r="C84" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="F84" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="85" spans="3:6">
       <c r="C85" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="F85" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="86" spans="3:6">
       <c r="C86" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="F86" t="s">
         <v>26</v>
@@ -4522,63 +4541,63 @@
     </row>
     <row r="87" spans="3:6">
       <c r="C87" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="F87" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="88" spans="3:6">
       <c r="C88" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="F88" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="89" spans="3:6">
       <c r="C89" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F89" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="90" spans="3:6">
       <c r="C90" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="F90" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="91" spans="3:6">
       <c r="C91" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="F91" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="92" spans="3:6">
       <c r="C92" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F92" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="93" spans="3:6">
       <c r="C93" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="F93" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="94" spans="3:6">
       <c r="C94" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F94" t="s">
         <v>26</v>
@@ -4586,71 +4605,71 @@
     </row>
     <row r="95" spans="3:6">
       <c r="C95" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="F95" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="96" spans="3:6">
       <c r="C96" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F96" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="97" spans="3:6">
       <c r="C97" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F97" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="98" spans="3:6">
       <c r="C98" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F98" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="99" spans="3:6">
       <c r="C99" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="F99" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="100" spans="3:6">
       <c r="C100" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F100" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="101" spans="3:6">
       <c r="C101" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="F101" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="102" spans="3:6">
       <c r="C102" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="F102" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="103" spans="3:6">
       <c r="C103" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="F103" t="s">
         <v>26</v>
@@ -4658,15 +4677,15 @@
     </row>
     <row r="104" spans="3:6">
       <c r="C104" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="F104" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="105" spans="3:6">
       <c r="C105" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="F105" t="s">
         <v>26</v>
@@ -4674,143 +4693,143 @@
     </row>
     <row r="106" spans="3:6">
       <c r="C106" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="F106" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="107" spans="3:6">
       <c r="C107" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="F107" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="108" spans="3:6">
       <c r="C108" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="F108" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="109" spans="3:6">
       <c r="C109" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="F109" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="110" spans="3:6">
       <c r="C110" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="F110" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="111" spans="3:6">
       <c r="C111" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="F111" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="112" spans="3:6">
       <c r="C112" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="F112" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="113" spans="3:6">
       <c r="C113" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="F113" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="114" spans="3:6">
       <c r="C114" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="F114" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="115" spans="3:6">
       <c r="C115" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="F115" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="116" spans="3:6">
       <c r="C116" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="F116" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="117" spans="3:6">
       <c r="C117" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="F117" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="118" spans="3:6">
       <c r="C118" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="F118" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="119" spans="3:6">
       <c r="C119" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F119" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="120" spans="3:6">
       <c r="C120" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="F120" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="121" spans="3:6">
       <c r="C121" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="F121" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="122" spans="3:6">
       <c r="C122" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="F122" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="123" spans="3:6">
       <c r="C123" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F123" t="s">
         <v>26</v>
@@ -4818,63 +4837,63 @@
     </row>
     <row r="124" spans="3:6">
       <c r="C124" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="F124" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="125" spans="3:6">
       <c r="C125" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F125" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
     <row r="126" spans="3:6">
       <c r="C126" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="F126" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="127" spans="3:6">
       <c r="C127" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="F127" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="128" spans="3:6">
       <c r="C128" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="F128" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="129" spans="3:6">
       <c r="C129" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="F129" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="130" spans="3:6">
       <c r="C130" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="F130" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="131" spans="3:6">
       <c r="C131" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="F131" t="s">
         <v>26</v>
@@ -4882,15 +4901,15 @@
     </row>
     <row r="132" spans="3:6">
       <c r="C132" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="F132" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="133" spans="3:6">
       <c r="C133" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F133" t="s">
         <v>26</v>
@@ -4898,23 +4917,23 @@
     </row>
     <row r="134" spans="3:6">
       <c r="C134" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="F134" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="135" spans="3:6">
       <c r="C135" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F135" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="136" spans="3:6">
       <c r="C136" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="F136" t="s">
         <v>26</v>
@@ -4922,31 +4941,31 @@
     </row>
     <row r="137" spans="3:6">
       <c r="C137" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="F137" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
     <row r="138" spans="3:6">
       <c r="C138" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="F138" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="139" spans="3:6">
       <c r="C139" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="F139" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="140" spans="3:6">
       <c r="C140" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F140" t="s">
         <v>26</v>
@@ -4954,71 +4973,71 @@
     </row>
     <row r="141" spans="3:6">
       <c r="C141" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="F141" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
     </row>
     <row r="142" spans="3:6">
       <c r="C142" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="F142" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="143" spans="3:6">
       <c r="C143" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="F143" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="144" spans="3:6">
       <c r="C144" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F144" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
     </row>
     <row r="145" spans="3:6">
       <c r="C145" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="F145" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
     </row>
     <row r="146" spans="3:6">
       <c r="C146" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="F146" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="147" spans="3:6">
       <c r="C147" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="F147" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="148" spans="3:6">
       <c r="C148" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="F148" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="149" spans="3:6">
       <c r="C149" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="F149" t="s">
         <v>26</v>
@@ -5026,191 +5045,191 @@
     </row>
     <row r="150" spans="3:6">
       <c r="C150" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="F150" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="151" spans="3:6">
       <c r="C151" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="F151" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="152" spans="3:6">
       <c r="C152" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="F152" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="153" spans="3:6">
       <c r="C153" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="F153" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="154" spans="3:6">
       <c r="C154" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="F154" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="155" spans="3:6">
       <c r="C155" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F155" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="156" spans="3:6">
       <c r="C156" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="F156" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="157" spans="3:6">
       <c r="C157" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="F157" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="158" spans="3:6">
       <c r="C158" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="F158" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
     </row>
     <row r="159" spans="3:6">
       <c r="C159" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="F159" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="160" spans="3:6">
       <c r="C160" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="F160" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="161" spans="3:6">
       <c r="C161" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="F161" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="162" spans="3:6">
       <c r="C162" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="F162" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
     </row>
     <row r="163" spans="3:6">
       <c r="C163" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F163" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="164" spans="3:6">
       <c r="C164" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F164" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="165" spans="3:6">
       <c r="C165" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="F165" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="166" spans="3:6">
       <c r="C166" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="F166" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
     </row>
     <row r="167" spans="3:6">
       <c r="C167" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="F167" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
     </row>
     <row r="168" spans="3:6">
       <c r="C168" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="F168" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
     </row>
     <row r="169" spans="3:6">
       <c r="C169" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="F169" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
     </row>
     <row r="170" spans="3:6">
       <c r="C170" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="F170" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
     </row>
     <row r="171" spans="3:6">
       <c r="C171" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="F171" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="172" spans="3:6">
       <c r="C172" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="F172" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
     </row>
     <row r="173" spans="3:6">
       <c r="C173" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="F173" t="s">
         <v>26</v>
@@ -5218,23 +5237,23 @@
     </row>
     <row r="174" spans="3:6">
       <c r="C174" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="F174" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="175" spans="3:6">
       <c r="C175" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="F175" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
     <row r="176" spans="3:6">
       <c r="C176" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="F176" t="s">
         <v>26</v>
@@ -5242,55 +5261,55 @@
     </row>
     <row r="177" spans="3:6">
       <c r="C177" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="F177" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="178" spans="3:6">
       <c r="C178" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="F178" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
     </row>
     <row r="179" spans="3:6">
       <c r="C179" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="F179" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="180" spans="3:6">
       <c r="C180" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="F180" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
     </row>
     <row r="181" spans="3:6">
       <c r="C181" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="F181" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="182" spans="3:6">
       <c r="C182" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="F182" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="183" spans="3:6">
       <c r="C183" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="F183" t="s">
         <v>26</v>
@@ -5298,23 +5317,23 @@
     </row>
     <row r="184" spans="3:6">
       <c r="C184" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="F184" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="185" spans="3:6">
       <c r="C185" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="F185" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
     </row>
     <row r="186" spans="3:6">
       <c r="C186" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="F186" t="s">
         <v>26</v>
@@ -5322,57 +5341,57 @@
     </row>
     <row r="187" spans="3:6">
       <c r="C187" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="F187" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="188" spans="3:6">
       <c r="C188" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="F188" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="189" spans="3:6">
       <c r="C189" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="F189" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="190" spans="3:6">
       <c r="C190" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="F190" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="191" spans="3:6">
       <c r="C191" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="F191" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
     </row>
     <row r="192" spans="3:6">
       <c r="F192" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
     <row r="193" spans="6:6">
       <c r="F193" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
     </row>
     <row r="194" spans="6:6">
       <c r="F194" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
     </row>
     <row r="195" spans="6:6">
@@ -5387,32 +5406,32 @@
     </row>
     <row r="197" spans="6:6">
       <c r="F197" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="198" spans="6:6">
       <c r="F198" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
     </row>
     <row r="199" spans="6:6">
       <c r="F199" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
     </row>
     <row r="200" spans="6:6">
       <c r="F200" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="201" spans="6:6">
       <c r="F201" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
     </row>
     <row r="202" spans="6:6">
       <c r="F202" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
     </row>
     <row r="203" spans="6:6">
@@ -5422,202 +5441,202 @@
     </row>
     <row r="204" spans="6:6">
       <c r="F204" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
     </row>
     <row r="205" spans="6:6">
       <c r="F205" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
     </row>
     <row r="206" spans="6:6">
       <c r="F206" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
     </row>
     <row r="207" spans="6:6">
       <c r="F207" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="208" spans="6:6">
       <c r="F208" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
     </row>
     <row r="209" spans="6:6">
       <c r="F209" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
     </row>
     <row r="210" spans="6:6">
       <c r="F210" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="211" spans="6:6">
       <c r="F211" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
     </row>
     <row r="212" spans="6:6">
       <c r="F212" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
     </row>
     <row r="213" spans="6:6">
       <c r="F213" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
     </row>
     <row r="214" spans="6:6">
       <c r="F214" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
     </row>
     <row r="215" spans="6:6">
       <c r="F215" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
     </row>
     <row r="216" spans="6:6">
       <c r="F216" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="217" spans="6:6">
       <c r="F217" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="218" spans="6:6">
       <c r="F218" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="219" spans="6:6">
       <c r="F219" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
     </row>
     <row r="220" spans="6:6">
       <c r="F220" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
     </row>
     <row r="221" spans="6:6">
       <c r="F221" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="222" spans="6:6">
       <c r="F222" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="223" spans="6:6">
       <c r="F223" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="224" spans="6:6">
       <c r="F224" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="225" spans="6:6">
       <c r="F225" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
     </row>
     <row r="226" spans="6:6">
       <c r="F226" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
     </row>
     <row r="227" spans="6:6">
       <c r="F227" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
     </row>
     <row r="228" spans="6:6">
       <c r="F228" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="229" spans="6:6">
       <c r="F229" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="230" spans="6:6">
       <c r="F230" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="231" spans="6:6">
       <c r="F231" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
     </row>
     <row r="232" spans="6:6">
       <c r="F232" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
     </row>
     <row r="233" spans="6:6">
       <c r="F233" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
     </row>
     <row r="234" spans="6:6">
       <c r="F234" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
     </row>
     <row r="235" spans="6:6">
       <c r="F235" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
     </row>
     <row r="236" spans="6:6">
       <c r="F236" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="237" spans="6:6">
       <c r="F237" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="238" spans="6:6">
       <c r="F238" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="239" spans="6:6">
       <c r="F239" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="240" spans="6:6">
       <c r="F240" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="241" spans="6:6">
       <c r="F241" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
     </row>
     <row r="242" spans="6:6">
       <c r="F242" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
     </row>
     <row r="243" spans="6:6">
       <c r="F243" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
   </sheetData>

</xml_diff>